<commit_message>
Removed entirely: ADC conversion latency input, pipeline stages input, effective initiation interval, pipeline fill/drain, streaming pipeline equations, and PE utilization.
Cycle model is now one line: Cycles per Batch = M (one row of activations streamed per cycle, per batch), Total Cycles = Batches × Cycles per Batch. No hardware detail beyond what you specified is baked in.

PSUM section now shows Required vs. Available directly, with a ✓ Fits / ❌ Overflow status cell (green/red conditional formatting) instead of a percentage — with the example inputs (196×160×160, 64 KB PSUM) it actually overflows at 65.08 KB required, which is a good demonstration that the check works.

Array Utilization is now just Arrays Used ÷ Total Arrays (averaged across batches), no PE-level utilization.

Dashboard is trimmed to exactly the five groups you listed: Hardware, Workload, Performance, Memory, Utilization — nothing extra.
</commit_message>
<xml_diff>
--- a/cim_architecture_estimator.xlsx
+++ b/cim_architecture_estimator.xlsx
@@ -62,7 +62,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Total independently-operable analog CIM array instances in the accelerator.</t>
+          <t xml:space="preserve">Total independently-operable CIM array instances in the accelerator.</t>
         </r>
       </text>
     </comment>
@@ -74,7 +74,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Bits per ADC conversion (per column readout).</t>
+          <t xml:space="preserve">Bits per ADC conversion (per column readout). Used only for reference; does not affect cycle/latency estimates in this first-order model.</t>
         </r>
       </text>
     </comment>
@@ -122,7 +122,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">e.g. number of input tokens / spatial positions streamed through the array.</t>
+          <t xml:space="preserve">Number of input tokens / spatial positions streamed through the array.</t>
         </r>
       </text>
     </comment>
@@ -159,30 +159,6 @@
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">Available on-chip partial-sum accumulator memory capacity.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B23" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Cycles for one ADC conversion (pipeline depth of the ADC readout path).</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B24" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">0 or blank = no pipelining assumed (ADC latency applied every cycle). &gt;0 spreads ADC latency across stages, reducing the effective initiation interval.</t>
         </r>
       </text>
     </comment>
@@ -204,7 +180,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Array Rows x Array Cols (assumption: a 32x32 array = 1024 PEs).</t>
+          <t xml:space="preserve">Array Rows x Array Cols. Assumption: one PE stores one weight (a 32x32 array = 1024 PEs).</t>
         </r>
       </text>
     </comment>
@@ -217,18 +193,6 @@
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">Assumption: one ADC per column of the array.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="A13" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Cycles between successive input rows being accepted. If pipeline stages &gt; 0, ADC latency is spread across stages (rounded up); otherwise the full ADC latency is charged per row.</t>
         </r>
       </text>
     </comment>
@@ -286,11 +250,23 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Assumption: arrays execute tiles in parallel; Batches = CEILING(Tiles / Arrays). Tiles that don't fit in one round are processed in a subsequent batch.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="A14" authorId="0">
+          <t xml:space="preserve">Batches = CEILING(Total Tiles / Number of Arrays). A batch is one round of computation, used only when there are more tiles than available arrays.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="A11" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Total Tiles / Batches — how many arrays are kept busy on average across all batches (the last batch may use fewer than the full array count).</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="A15" authorId="0">
       <text>
         <r>
           <rPr>
@@ -320,7 +296,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Classic pipeline latency: (M-1) x Initiation Interval + ADC latency (fill + drain), assuming activations for a tile are streamed one row per II cycles across arrays operating in parallel.</t>
+          <t xml:space="preserve">First-order assumption: one activation row (of M) is streamed and processed per clock cycle, in parallel across all arrays in the batch.</t>
         </r>
       </text>
     </comment>
@@ -332,7 +308,19 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Batches are executed sequentially; tiles within a batch run in parallel across arrays.</t>
+          <t xml:space="preserve">Batches x Cycles per Batch. Batches run sequentially; tiles within a batch run in parallel across arrays.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="A11" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Total Cycles / Clock Frequency.</t>
         </r>
       </text>
     </comment>
@@ -368,19 +356,19 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Useful MACs performed / (Total PEs x Total cycles) — fraction of total PE-cycle capacity doing real work.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="A20" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Tiles actually needed / (Batches x Arrays) — fraction of array-slots used (a partially-filled final batch lowers this).</t>
+          <t xml:space="preserve">Arrays Used / Total Arrays (averaged across batches).</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="A23" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Assumption: accumulator width = weight bits + activation bits + log2(array rows), to bound worst-case growth from summing K partial products within one tile.</t>
         </r>
       </text>
     </comment>
@@ -392,19 +380,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Assumption: accumulator width = weight bits + activation bits + log2(array rows), to bound worst-case growth from summing K partial products.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="A25" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">M x N output elements x accumulator width, converted to KB. Assumes the full output tile is resident before write-back.</t>
+          <t xml:space="preserve">M x N output elements x accumulator width, converted to KB. Assumes the full output tile's accumulators are resident before write-back.</t>
         </r>
       </text>
     </comment>
@@ -416,7 +392,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Required PSUM storage / configured PSUM capacity. &gt;100% means the configured PSUM memory is undersized for this workload.</t>
+          <t xml:space="preserve">Fits if Required PSUM Storage &lt;= Available PSUM Storage, otherwise Overflow.</t>
         </r>
       </text>
     </comment>
@@ -425,12 +401,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="117">
-  <si>
-    <t xml:space="preserve">CIM Architecture Estimator — User Inputs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Edit only the yellow cells below (blue text = editable input). All other sheets compute automatically from these values.</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="118">
+  <si>
+    <t xml:space="preserve">CIM First-Order Architectural Estimator — User Inputs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Edit only the yellow cells below. All other sheets compute automatically from these values.</t>
   </si>
   <si>
     <t xml:space="preserve">Array &amp; System Configuration</t>
@@ -502,135 +478,117 @@
     <t xml:space="preserve">Matrix Dimension N (cols of weight matrix)</t>
   </si>
   <si>
-    <t xml:space="preserve">Memory &amp; Pipeline Configuration</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PSUM Memory Size (capacity)</t>
+    <t xml:space="preserve">Memory Configuration</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PSUM Memory Size (available capacity)</t>
   </si>
   <si>
     <t xml:space="preserve">KB</t>
   </si>
   <si>
-    <t xml:space="preserve">ADC Conversion Latency</t>
+    <t xml:space="preserve">Derived Hardware Parameters</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All cells below are computed with formulas from 'User Inputs'. No manual edits needed.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Processing Elements &amp; ADCs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Metric</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Formula / Notes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PEs per Array</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PEs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total Number of PEs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Number of ADCs per Array</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ADCs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total Number of ADCs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Workload Mapping</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maps the (M x K) . (K x N) matrix multiplication onto the array grid. Arrays execute tiles in parallel; batches only occur if there are more tiles than arrays.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiling</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiles along K (contraction dim)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tiles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiles along N (output dim)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total Number of Tiles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Number of Arrays Available</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Number of Batches Required</t>
+  </si>
+  <si>
+    <t xml:space="preserve">batches</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Average Arrays Used per Batch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compute Volume</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total MAC Operations</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MACs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Performance Estimation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">First-order estimate only. One clock cycle streams one row of M through a tile; no pipeline fill/drain, ADC settling, or timing overlap is modeled.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cycle Estimation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cycles per Batch</t>
   </si>
   <si>
     <t xml:space="preserve">cycles</t>
   </si>
   <si>
-    <t xml:space="preserve">Number of Pipeline Stages (optional)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">stages</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Derived Hardware Parameters</t>
-  </si>
-  <si>
-    <t xml:space="preserve">All cells below are computed with formulas from 'User Inputs'. No manual edits needed.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Processing Elements &amp; ADCs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Metric</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Formula / Notes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PEs per Array</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PEs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total Number of PEs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Number of ADCs per Array</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ADCs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total Number of ADCs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Derived Timing Parameters</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Effective Initiation Interval (II)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cycles/row</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Clock Period</t>
+    <t xml:space="preserve">Total Estimated Execution Cycles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Latency &amp; Throughput</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estimated Latency</t>
   </si>
   <si>
     <t xml:space="preserve">s</t>
   </si>
   <si>
-    <t xml:space="preserve">Workload Mapping</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Maps the (M x K) . (K x N) matrix multiplication onto the array grid.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tiling</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tiles along K (contraction dim)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tiles</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tiles along N (output dim)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total Number of Tiles</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Number of Arrays Available</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Number of Batches Required</t>
-  </si>
-  <si>
-    <t xml:space="preserve">batches</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Compute Volume</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total MAC Operations</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MACs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Performance Estimation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Architectural (not device-physics) estimate of cycles, latency, throughput and utilization.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cycle Estimation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cycles per Tile Pass (all M rows through one tile set)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total Estimated Execution Cycles</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Latency &amp; Throughput</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Estimated Latency</t>
-  </si>
-  <si>
     <t xml:space="preserve">ms</t>
   </si>
   <si>
@@ -646,70 +604,91 @@
     <t xml:space="preserve">TOPS</t>
   </si>
   <si>
+    <t xml:space="preserve">Array Utilization</t>
+  </si>
+  <si>
+    <t xml:space="preserve">%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PSUM Memory</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estimated PSUM Accumulator Width</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Required PSUM Storage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Available PSUM Storage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Status</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Summary Dashboard — CIM First-Order Estimate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Live links to the calculation sheets. Architecture-level estimate only — see the Assumptions sheet.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hardware</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Array Size</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Number of Arrays</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total PEs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total ADCs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Workload</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Matrix Size (M x K x N)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total Tiles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total Batches</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Performance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estimated Cycles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Latency</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Throughput</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Memory</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Required PSUM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Available PSUM</t>
+  </si>
+  <si>
     <t xml:space="preserve">Utilization</t>
   </si>
   <si>
-    <t xml:space="preserve">PE Utilization</t>
-  </si>
-  <si>
-    <t xml:space="preserve">%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Array Utilization</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PSUM Storage</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Estimated PSUM Accumulator Width</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Estimated PSUM Storage Requirement</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PSUM Memory Utilization</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Summary Dashboard — CIM Accelerator Architecture Estimate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">All values below are live links to the calculation sheets.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Number of Arrays</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total PEs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total ADCs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Matrix Size (M x K x N)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total Tiles</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total Batches</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Estimated Cycles</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Throughput</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PSUM Utilization</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Note: this is an architectural estimator (cycles, latency, throughput, utilization). It does not model analog device physics (settling time, noise, IR drop, etc.). See the Assumptions sheet for every modeling assumption.</t>
+    <t xml:space="preserve">Note: this is a first-order architectural estimator (fit, tiles, batches, array utilization, approximate cycles/latency/throughput, PSUM fit check). It does not model pipeline timing, ADC settling, analog non-idealities, routing delays, or RTL-level behavior. See the Assumptions sheet.</t>
   </si>
   <si>
     <t xml:space="preserve">Assumptions</t>
   </si>
   <si>
-    <t xml:space="preserve">This workbook is an architectural estimator for throughput, latency, utilization and workload mapping. It does NOT model analog device physics (IR drop, settling time, noise margins, thermal effects, etc.).</t>
+    <t xml:space="preserve">This workbook is a first-order architecture-level estimator only. It exists to sanity-check whether a workload fits an architecture before building the detailed cim_sim Python simulator.</t>
   </si>
   <si>
     <t xml:space="preserve">#</t>
@@ -721,61 +700,61 @@
     <t xml:space="preserve">One ADC is assigned per column of a CIM array (ADCs per array = Array Cols).</t>
   </si>
   <si>
-    <t xml:space="preserve">A 32x32 array contains 1024 Processing Elements (PEs per array = Array Rows x Array Cols).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The (M x K) . (K x N) matrix multiplication is tiled spatially: K (contraction dim) is tiled by the array's row dimension; N (output dim) is tiled by the array's column dimension. M (tokens/rows) is streamed temporally through a tile, not tiled spatially.</t>
+    <t xml:space="preserve">One PE stores one weight; a 32x32 array therefore contains 1024 PEs (PEs per array = Array Rows x Array Cols).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The (M x K) . (K x N) matrix multiplication is partitioned into tiles sized to the array: K (contraction dim) is tiled by Array Rows, N (output dim) is tiled by Array Cols. M (tokens/rows) is streamed through a tile rather than tiled spatially.</t>
   </si>
   <si>
     <t xml:space="preserve">Total tiles required = CEILING(K / Array Rows) x CEILING(N / Array Cols).</t>
   </si>
   <si>
-    <t xml:space="preserve">All CIM arrays execute their assigned tile in parallel within a batch.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Batches required = CEILING(Total Tiles / Number of Arrays) — tiles that do not fit in one parallel round are processed in a subsequent batch, run sequentially.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cycles per tile pass follow a simple pipeline model: (M - 1) x Initiation Interval + ADC Conversion Latency (classic fill + drain latency), assuming one input row is accepted every 'Initiation Interval' cycles.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Initiation Interval = CEILING(ADC Latency / Pipeline Stages) if Pipeline Stages &gt; 0, otherwise the full ADC Conversion Latency is charged every cycle (no pipelining).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total estimated cycles = Batches x Cycles per tile pass (batches are sequential; tiles within a batch are parallel across arrays).</t>
+    <t xml:space="preserve">Arrays execute their assigned tile in parallel — all arrays active in a batch work simultaneously.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Batches occur only when the number of tiles exceeds the number of available arrays: Batches = CEILING(Total Tiles / Number of Arrays). One batch = one round of computation.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">First-order cycle model: one row of the M dimension is processed per clock cycle, per batch (Cycles per Batch = M). No pipeline fill/drain, initiation interval, ADC settling, or cycle-level timing overlap is modeled.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total Estimated Execution Cycles = Batches x Cycles per Batch (batches run sequentially; tiles within a batch run in parallel across arrays).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estimated Latency = Total Cycles / Clock Frequency. This is a rough architectural estimate, not a cycle-accurate or RTL timing result.</t>
   </si>
   <si>
     <t xml:space="preserve">1 MAC (multiply-accumulate) is counted as 2 operations (1 multiply + 1 add) when converting MACs/s to Ops/s and TOPS.</t>
   </si>
   <si>
-    <t xml:space="preserve">PE Utilization = Total useful MAC operations / (Total PEs x Total estimated cycles) — the fraction of total available PE-cycle capacity doing real work; a partially-filled final tile or batch will lower this.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Array Utilization = Total Tiles / (Batches x Number of Arrays) — the fraction of array-slots actually used across all batches.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Estimated PSUM accumulator width = Weight Precision + Activation Precision + log2(Array Rows), rounded up — a conservative bound on bit growth from summing partial products across the contraction dimension of one tile.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Estimated PSUM storage requirement = M x N x (PSUM accumulator width in bits) / 8 / 1024, i.e. enough KB to hold the full M x N output tile's accumulators before write-back to on-chip memory.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PSUM Memory Utilization compares the estimated requirement against the user-specified PSUM capacity input; values above 100% indicate the configured PSUM memory is undersized and results would need to be spilled or tiled further.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Clock frequency is assumed constant (no dynamic voltage/frequency scaling) and applies uniformly to all arrays and the digital control/pipeline logic.</t>
+    <t xml:space="preserve">Array Utilization = Arrays Used / Total Arrays, averaged across all batches (Total Tiles / Batches / Total Arrays). It reflects how fully the array grid is occupied, not compute efficiency within a tile.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estimated PSUM accumulator width = Weight Precision + Activation Precision + log2(Array Rows), rounded up — a simple bound on bit growth from summing partial products across the contraction dimension of one tile.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Required PSUM Storage = M x N x (PSUM accumulator width in bits) / 8 / 1024 — enough KB to hold the full M x N output tile's accumulators before write-back.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fit is checked by direct comparison: Required PSUM Storage vs. Available PSUM Storage (the user-specified capacity). 'Overflow' means the configured PSUM memory is too small for this workload as mapped; utilization percentage above 100% is intentionally not shown, since Fit/Overflow is the more actionable signal.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ADC resolution is recorded as a configuration input for downstream reference (e.g. accuracy/power modeling) but does not affect the cycle, latency, or throughput formulas in this first-order model.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clock frequency is assumed constant across the whole run (no dynamic voltage/frequency scaling) and applies uniformly to all arrays.</t>
   </si>
   <si>
     <t xml:space="preserve">All arrays are assumed identical in size, precision, and timing (no heterogeneous array configurations).</t>
   </si>
   <si>
-    <t xml:space="preserve">Weight-write / reprogramming time for the analog CIM cells (e.g. for dynamic weights) is NOT included in this cycle/latency estimate — this model targets execution-cycle throughput only.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ADC resolution, weight precision and activation precision are tracked as configuration inputs but do not independently affect the cycle-count formulas above beyond their role in PSUM width; they are provided for downstream accuracy/power modeling outside this workbook.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">This workbook is intended to validate architecture-level throughput/latency/utilization trends before implementing the detailed cim_sim Python simulator — it is not a substitute for cycle-accurate or SPICE-level simulation.</t>
+    <t xml:space="preserve">Weight-write / reprogramming time for the CIM cells (e.g. for dynamic weights) is NOT included in this estimate.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This spreadsheet estimates architecture-level performance only. It does not model analog non-idealities, ADC settling time, routing delays, pipeline effects, memory bandwidth limitations, or RTL-level timing.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This workbook is intended to sanity-check architecture-level fit, tiling, and rough performance trends before implementing the detailed cim_sim Python simulator — it is not a substitute for cycle-accurate or SPICE-level simulation.</t>
   </si>
 </sst>
 </file>
@@ -786,13 +765,13 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0"/>
     <numFmt numFmtId="166" formatCode="General"/>
-    <numFmt numFmtId="167" formatCode="0.00E+00"/>
-    <numFmt numFmtId="168" formatCode="0.000000"/>
-    <numFmt numFmtId="169" formatCode="#,##0.000"/>
+    <numFmt numFmtId="167" formatCode="0.000000"/>
+    <numFmt numFmtId="168" formatCode="#,##0.000"/>
+    <numFmt numFmtId="169" formatCode="0.00E+00"/>
     <numFmt numFmtId="170" formatCode="#,##0.00"/>
     <numFmt numFmtId="171" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="17">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -884,6 +863,14 @@
     </font>
     <font>
       <b val="true"/>
+      <sz val="14"/>
+      <color rgb="FF1F4E78"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
       <sz val="16"/>
       <color rgb="FF1F4E78"/>
       <name val="Arial"/>
@@ -894,6 +881,14 @@
       <b val="true"/>
       <sz val="13"/>
       <color rgb="FF1F4E78"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="16"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -921,7 +916,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFD9E1F2"/>
-        <bgColor rgb="FFCCFFFF"/>
+        <bgColor rgb="FFC6EFCE"/>
       </patternFill>
     </fill>
     <fill>
@@ -980,7 +975,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="28">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1041,15 +1036,19 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1057,15 +1056,23 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="170" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1090,6 +1097,30 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <dxfs count="2">
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -1100,7 +1131,7 @@
       <rgbColor rgb="FFFFFF00"/>
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FF00FFFF"/>
-      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF9C0006"/>
       <rgbColor rgb="FF008000"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FF808000"/>
@@ -1126,12 +1157,12 @@
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FF00CCFF"/>
       <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FFCCFFCC"/>
+      <rgbColor rgb="FFC6EFCE"/>
       <rgbColor rgb="FFFFFF99"/>
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFFFCC99"/>
+      <rgbColor rgb="FFFFC7CE"/>
       <rgbColor rgb="FF2E75B6"/>
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
@@ -1142,7 +1173,7 @@
       <rgbColor rgb="FF969696"/>
       <rgbColor rgb="FF003366"/>
       <rgbColor rgb="FF339966"/>
-      <rgbColor rgb="FF003300"/>
+      <rgbColor rgb="FF006100"/>
       <rgbColor rgb="FF333300"/>
       <rgbColor rgb="FF993300"/>
       <rgbColor rgb="FF993366"/>
@@ -1333,7 +1364,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
@@ -1543,28 +1574,6 @@
       </c>
       <c r="C22" s="7" t="s">
         <v>27</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="B23" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="C23" s="7" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="B24" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="C24" s="7" t="s">
-        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -1591,7 +1600,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
@@ -1602,7 +1611,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1610,7 +1619,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1618,7 +1627,7 @@
     </row>
     <row r="4" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
@@ -1626,7 +1635,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>4</v>
@@ -1635,109 +1644,62 @@
         <v>5</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="B6" s="8" t="n">
         <f aca="false">'User Inputs'!B6*'User Inputs'!B7</f>
         <v>1024</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="B7" s="8" t="n">
         <f aca="false">B6*'User Inputs'!B8</f>
         <v>16384</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="B8" s="8" t="n">
         <f aca="false">'User Inputs'!B7</f>
         <v>32</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="B9" s="8" t="n">
         <f aca="false">B8*'User Inputs'!B8</f>
         <v>512</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="B13" s="9" t="n">
-        <f aca="false">IF('User Inputs'!B24&gt;0,CEILING('User Inputs'!B23/'User Inputs'!B24,1),'User Inputs'!B23)</f>
-        <v>3</v>
-      </c>
-      <c r="C13" s="7" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="B14" s="10" t="n">
-        <f aca="false">1/('User Inputs'!B12*1000000)</f>
-        <v>2E-009</v>
-      </c>
-      <c r="C14" s="7" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="3">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="A4:D4"/>
-    <mergeCell ref="A11:D11"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1755,7 +1717,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
@@ -1766,15 +1728,15 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1782,7 +1744,7 @@
     </row>
     <row r="4" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
@@ -1790,7 +1752,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>4</v>
@@ -1799,48 +1761,48 @@
         <v>5</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="B6" s="9" t="n">
         <f aca="false">CEILING('User Inputs'!B17/'User Inputs'!B6,1)</f>
         <v>5</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>52</v>
+        <v>43</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
       <c r="B7" s="9" t="n">
         <f aca="false">CEILING('User Inputs'!B18/'User Inputs'!B7,1)</f>
         <v>5</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>52</v>
+        <v>43</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="B8" s="9" t="n">
         <f aca="false">B6*B7</f>
         <v>25</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>52</v>
+        <v>43</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="B9" s="9" t="n">
         <f aca="false">'User Inputs'!B8</f>
@@ -1852,48 +1814,60 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>56</v>
+        <v>47</v>
       </c>
       <c r="B10" s="9" t="n">
         <f aca="false">CEILING(B8/B9,1)</f>
         <v>2</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="B12" s="3"/>
-      <c r="C12" s="3"/>
-      <c r="D12" s="3"/>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="B13" s="4" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="B11" s="9" t="n">
+        <f aca="false">B8/B10</f>
+        <v>12.5</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="B13" s="3"/>
+      <c r="C13" s="3"/>
+      <c r="D13" s="3"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B14" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C14" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="D13" s="4" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="B14" s="8" t="n">
+      <c r="D14" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B15" s="8" t="n">
         <f aca="false">'User Inputs'!B16*'User Inputs'!B17*'User Inputs'!B18</f>
         <v>5017600</v>
       </c>
-      <c r="C14" s="7" t="s">
-        <v>60</v>
+      <c r="C15" s="7" t="s">
+        <v>52</v>
       </c>
     </row>
   </sheetData>
@@ -1901,7 +1875,7 @@
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="A4:D4"/>
-    <mergeCell ref="A12:D12"/>
+    <mergeCell ref="A13:D13"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1930,15 +1904,15 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>62</v>
+        <v>54</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1946,7 +1920,7 @@
     </row>
     <row r="4" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
@@ -1954,7 +1928,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>4</v>
@@ -1963,36 +1937,36 @@
         <v>5</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="B6" s="8" t="n">
-        <f aca="false">('User Inputs'!B16-1)*'Derived Hardware Parameters'!B13+'User Inputs'!B23</f>
-        <v>595</v>
+        <f aca="false">'User Inputs'!B16</f>
+        <v>196</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>29</v>
+        <v>57</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="B7" s="8" t="n">
         <f aca="false">'Workload Mapping'!B10*B6</f>
-        <v>1190</v>
+        <v>392</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>29</v>
+        <v>57</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
@@ -2000,7 +1974,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>4</v>
@@ -2009,72 +1983,72 @@
         <v>5</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="B11" s="11" t="n">
+        <v>60</v>
+      </c>
+      <c r="B11" s="10" t="n">
         <f aca="false">B7/('User Inputs'!B12*1000000)</f>
-        <v>2.38E-006</v>
+        <v>7.84E-007</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>47</v>
+        <v>61</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="B12" s="12" t="n">
+        <v>60</v>
+      </c>
+      <c r="B12" s="11" t="n">
         <f aca="false">B11*1000</f>
-        <v>0.00238</v>
+        <v>0.000784</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="B13" s="10" t="n">
-        <f aca="false">'Workload Mapping'!B14/B11</f>
-        <v>2108235294117.65</v>
+        <v>63</v>
+      </c>
+      <c r="B13" s="12" t="n">
+        <f aca="false">'Workload Mapping'!B15/B11</f>
+        <v>6400000000000</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="B14" s="10" t="n">
+        <v>63</v>
+      </c>
+      <c r="B14" s="12" t="n">
         <f aca="false">B13*2</f>
-        <v>4216470588235.29</v>
+        <v>12800000000000</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="B15" s="13" t="n">
         <f aca="false">B14/1000000000000</f>
-        <v>4.21647058823529</v>
+        <v>12.8</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
@@ -2082,7 +2056,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="B18" s="4" t="s">
         <v>4</v>
@@ -2091,74 +2065,74 @@
         <v>5</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="B19" s="14" t="n">
-        <f aca="false">'Workload Mapping'!B14/('Derived Hardware Parameters'!B7*B7)</f>
-        <v>0.257352941176471</v>
+        <f aca="false">'Workload Mapping'!B11/'Workload Mapping'!B9</f>
+        <v>0.78125</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="B20" s="14" t="n">
-        <f aca="false">'Workload Mapping'!B8/('Workload Mapping'!B10*'Workload Mapping'!B9)</f>
-        <v>0.78125</v>
-      </c>
-      <c r="C20" s="7" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="B22" s="3"/>
-      <c r="C22" s="3"/>
-      <c r="D22" s="3"/>
+        <v>68</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="B21" s="3"/>
+      <c r="C21" s="3"/>
+      <c r="D21" s="3"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="B23" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C23" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="D23" s="4" t="s">
-        <v>36</v>
+      <c r="A23" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="B23" s="8" t="n">
+        <f aca="false">'User Inputs'!B10+'User Inputs'!B11+ROUNDUP(LOG('User Inputs'!B6,2),0)</f>
+        <v>17</v>
+      </c>
+      <c r="C23" s="7" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="B24" s="8" t="n">
-        <f aca="false">'User Inputs'!B10+'User Inputs'!B11+ROUNDUP(LOG('User Inputs'!B6,2),0)</f>
-        <v>17</v>
+        <v>71</v>
+      </c>
+      <c r="B24" s="13" t="n">
+        <f aca="false">'User Inputs'!B16*'User Inputs'!B18*B23/8/1024</f>
+        <v>65.078125</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>14</v>
+        <v>27</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="B25" s="13" t="n">
-        <f aca="false">'User Inputs'!B16*'User Inputs'!B18*B24/8/1024</f>
-        <v>65.078125</v>
+        <v>72</v>
+      </c>
+      <c r="B25" s="9" t="n">
+        <f aca="false">'User Inputs'!B22</f>
+        <v>64</v>
       </c>
       <c r="C25" s="7" t="s">
         <v>27</v>
@@ -2166,15 +2140,13 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="B26" s="14" t="n">
-        <f aca="false">B25/'User Inputs'!B22</f>
-        <v>1.016845703125</v>
-      </c>
-      <c r="C26" s="7" t="s">
-        <v>75</v>
-      </c>
+        <v>73</v>
+      </c>
+      <c r="B26" s="15" t="str">
+        <f aca="false">IF(B24&lt;=B25,"Fits","Overflow")</f>
+        <v>Overflow</v>
+      </c>
+      <c r="C26" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -2183,7 +2155,7 @@
     <mergeCell ref="A4:D4"/>
     <mergeCell ref="A9:D9"/>
     <mergeCell ref="A17:D17"/>
-    <mergeCell ref="A22:D22"/>
+    <mergeCell ref="A21:D21"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -2201,18 +2173,18 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="22"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2220,153 +2192,236 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>82</v>
+        <v>75</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="15" t="s">
-        <v>83</v>
-      </c>
-      <c r="B4" s="15" t="s">
-        <v>84</v>
-      </c>
-      <c r="C4" s="15" t="s">
-        <v>85</v>
-      </c>
-      <c r="D4" s="15" t="s">
-        <v>86</v>
-      </c>
+      <c r="A4" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
     </row>
     <row r="5" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="16" t="n">
+      <c r="A5" s="16" t="s">
+        <v>77</v>
+      </c>
+      <c r="B5" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="C5" s="16" t="s">
+        <v>79</v>
+      </c>
+      <c r="D5" s="16" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="17" t="str">
+        <f aca="false">'User Inputs'!B6&amp;" x "&amp;'User Inputs'!B7</f>
+        <v>32 x 32</v>
+      </c>
+      <c r="B6" s="18" t="n">
         <f aca="false">'User Inputs'!B8</f>
         <v>16</v>
       </c>
-      <c r="B5" s="16" t="n">
+      <c r="C6" s="18" t="n">
         <f aca="false">'Derived Hardware Parameters'!B7</f>
         <v>16384</v>
       </c>
-      <c r="C5" s="16" t="n">
+      <c r="D6" s="18" t="n">
         <f aca="false">'Derived Hardware Parameters'!B9</f>
         <v>512</v>
       </c>
-      <c r="D5" s="17" t="str">
+    </row>
+    <row r="7" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B7" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="D7" s="19" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+    </row>
+    <row r="9" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="16" t="s">
+        <v>82</v>
+      </c>
+      <c r="B9" s="16" t="s">
+        <v>83</v>
+      </c>
+      <c r="C9" s="16" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="20" t="str">
         <f aca="false">'User Inputs'!B16&amp;" x "&amp;'User Inputs'!B17&amp;" x "&amp;'User Inputs'!B18</f>
         <v>196 x 160 x 160</v>
       </c>
-    </row>
-    <row r="6" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6" s="18" t="s">
-        <v>38</v>
-      </c>
-      <c r="C6" s="18" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="B7" s="15" t="s">
-        <v>88</v>
-      </c>
-      <c r="C7" s="15" t="s">
-        <v>89</v>
-      </c>
-      <c r="D7" s="15" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="16" t="n">
+      <c r="B10" s="18" t="n">
         <f aca="false">'Workload Mapping'!B8</f>
         <v>25</v>
       </c>
-      <c r="B8" s="16" t="n">
+      <c r="C10" s="18" t="n">
         <f aca="false">'Workload Mapping'!B10</f>
         <v>2</v>
       </c>
-      <c r="C8" s="16" t="n">
+    </row>
+    <row r="11" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B11" s="19" t="s">
+        <v>43</v>
+      </c>
+      <c r="C11" s="19" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B12" s="3"/>
+      <c r="C12" s="3"/>
+      <c r="D12" s="3"/>
+    </row>
+    <row r="13" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="16" t="s">
+        <v>86</v>
+      </c>
+      <c r="B13" s="16" t="s">
+        <v>87</v>
+      </c>
+      <c r="C13" s="16" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="18" t="n">
         <f aca="false">'Performance Estimation'!B7</f>
-        <v>1190</v>
-      </c>
-      <c r="D8" s="19" t="n">
+        <v>392</v>
+      </c>
+      <c r="B14" s="21" t="n">
         <f aca="false">'Performance Estimation'!B12</f>
-        <v>0.00238</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="18" t="s">
-        <v>52</v>
-      </c>
-      <c r="B9" s="18" t="s">
+        <v>0.000784</v>
+      </c>
+      <c r="C14" s="22" t="n">
+        <f aca="false">'Performance Estimation'!B15</f>
+        <v>12.8</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="19" t="s">
         <v>57</v>
       </c>
-      <c r="C9" s="18" t="s">
-        <v>29</v>
-      </c>
-      <c r="D9" s="18" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="15" t="s">
+      <c r="B15" s="19" t="s">
+        <v>62</v>
+      </c>
+      <c r="C15" s="19" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="B16" s="3"/>
+      <c r="C16" s="3"/>
+      <c r="D16" s="3"/>
+    </row>
+    <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="16" t="s">
         <v>90</v>
       </c>
-      <c r="B10" s="15" t="s">
-        <v>74</v>
-      </c>
-      <c r="C10" s="15" t="s">
-        <v>76</v>
-      </c>
-      <c r="D10" s="15" t="s">
+      <c r="B17" s="16" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="11" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="20" t="n">
-        <f aca="false">'Performance Estimation'!B15</f>
-        <v>4.21647058823529</v>
-      </c>
-      <c r="B11" s="21" t="n">
+      <c r="C17" s="16" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="22" t="n">
+        <f aca="false">'Performance Estimation'!B24</f>
+        <v>65.078125</v>
+      </c>
+      <c r="B18" s="22" t="n">
+        <f aca="false">'Performance Estimation'!B25</f>
+        <v>64</v>
+      </c>
+      <c r="C18" s="23" t="str">
+        <f aca="false">IF('Performance Estimation'!B26="Fits","✓ Fits","❌ Overflow")</f>
+        <v>❌ Overflow</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="19" t="s">
+        <v>27</v>
+      </c>
+      <c r="B19" s="19" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="B20" s="3"/>
+      <c r="C20" s="3"/>
+      <c r="D20" s="3"/>
+    </row>
+    <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="16" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="24" t="n">
         <f aca="false">'Performance Estimation'!B19</f>
-        <v>0.257352941176471</v>
-      </c>
-      <c r="C11" s="21" t="n">
-        <f aca="false">'Performance Estimation'!B20</f>
         <v>0.78125</v>
       </c>
-      <c r="D11" s="21" t="n">
-        <f aca="false">'Performance Estimation'!B26</f>
-        <v>1.016845703125</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="18" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="22" t="s">
-        <v>92</v>
-      </c>
-      <c r="B14" s="22"/>
-      <c r="C14" s="22"/>
-      <c r="D14" s="22"/>
+    </row>
+    <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="24" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="25" t="s">
+        <v>93</v>
+      </c>
+      <c r="B24" s="25"/>
+      <c r="C24" s="25"/>
+      <c r="D24" s="25"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="8">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A14:D14"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A8:D8"/>
+    <mergeCell ref="A12:D12"/>
+    <mergeCell ref="A16:D16"/>
+    <mergeCell ref="A20:D20"/>
+    <mergeCell ref="A24:D24"/>
   </mergeCells>
+  <conditionalFormatting sqref="C18">
+    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>ISNUMBER(SEARCH("Overflow",C18))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>ISNUMBER(SEARCH("Fits",C18))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -2391,182 +2446,182 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B1" s="1"/>
     </row>
     <row r="2" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="22" t="s">
-        <v>94</v>
-      </c>
-      <c r="B2" s="22"/>
+      <c r="A2" s="25" t="s">
+        <v>95</v>
+      </c>
+      <c r="B2" s="25"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="23" t="n">
+      <c r="A5" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="24" t="s">
-        <v>97</v>
+      <c r="B5" s="27" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="23" t="n">
+      <c r="A6" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="24" t="s">
-        <v>98</v>
+      <c r="B6" s="27" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="23" t="n">
+      <c r="A7" s="26" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="24" t="s">
-        <v>99</v>
+      <c r="B7" s="27" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="23" t="n">
+      <c r="A8" s="26" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="24" t="s">
-        <v>100</v>
+      <c r="B8" s="27" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="23" t="n">
+      <c r="A9" s="26" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="24" t="s">
-        <v>101</v>
+      <c r="B9" s="27" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="23" t="n">
+      <c r="A10" s="26" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="24" t="s">
-        <v>102</v>
+      <c r="B10" s="27" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="23" t="n">
+      <c r="A11" s="26" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="24" t="s">
-        <v>103</v>
+      <c r="B11" s="27" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="23" t="n">
+      <c r="A12" s="26" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="24" t="s">
-        <v>104</v>
+      <c r="B12" s="27" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="23" t="n">
+      <c r="A13" s="26" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="24" t="s">
-        <v>105</v>
+      <c r="B13" s="27" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="23" t="n">
+      <c r="A14" s="26" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="24" t="s">
-        <v>106</v>
+      <c r="B14" s="27" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="23" t="n">
+      <c r="A15" s="26" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="24" t="s">
-        <v>107</v>
+      <c r="B15" s="27" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="23" t="n">
+      <c r="A16" s="26" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="24" t="s">
-        <v>108</v>
+      <c r="B16" s="27" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="23" t="n">
+      <c r="A17" s="26" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="24" t="s">
-        <v>109</v>
+      <c r="B17" s="27" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="23" t="n">
+      <c r="A18" s="26" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="24" t="s">
-        <v>110</v>
+      <c r="B18" s="27" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="23" t="n">
+      <c r="A19" s="26" t="n">
         <v>15</v>
       </c>
-      <c r="B19" s="24" t="s">
-        <v>111</v>
+      <c r="B19" s="27" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="23" t="n">
+      <c r="A20" s="26" t="n">
         <v>16</v>
       </c>
-      <c r="B20" s="24" t="s">
-        <v>112</v>
+      <c r="B20" s="27" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="23" t="n">
+      <c r="A21" s="26" t="n">
         <v>17</v>
       </c>
-      <c r="B21" s="24" t="s">
-        <v>113</v>
+      <c r="B21" s="27" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="23" t="n">
+      <c r="A22" s="26" t="n">
         <v>18</v>
       </c>
-      <c r="B22" s="24" t="s">
-        <v>114</v>
+      <c r="B22" s="27" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="23" t="n">
+      <c r="A23" s="26" t="n">
         <v>19</v>
       </c>
-      <c r="B23" s="24" t="s">
-        <v>115</v>
+      <c r="B23" s="27" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="23" t="n">
+      <c r="A24" s="26" t="n">
         <v>20</v>
       </c>
-      <c r="B24" s="24" t="s">
-        <v>116</v>
+      <c r="B24" s="27" t="s">
+        <v>117</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fixed the psum accumulator width formula. Now it considers accumulation across the K depth tiles, instead of one 32. psum memory is enough to hold the M x N (number of tokens x number of weight columns) outputs.
</commit_message>
<xml_diff>
--- a/cim_architecture_estimator.xlsx
+++ b/cim_architecture_estimator.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\THESIS\CIM_Soc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E642B4C-B23B-4F89-A279-44171280F31B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C42E85C-E293-45F5-8FAC-140F9F25FABB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-109" yWindow="-109" windowWidth="26301" windowHeight="16520" tabRatio="796" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1481,7 +1481,7 @@
         <v>24</v>
       </c>
       <c r="B22" s="7">
-        <v>64</v>
+        <v>128</v>
       </c>
       <c r="C22" s="8" t="s">
         <v>25</v>
@@ -1994,8 +1994,8 @@
         <v>68</v>
       </c>
       <c r="B23" s="9">
-        <f>'User Inputs'!B10+'User Inputs'!B11+ROUNDUP(LOG('User Inputs'!B6,2),0)</f>
-        <v>17</v>
+        <f>'User Inputs'!B10+'User Inputs'!B11+ROUNDUP(LOG('User Inputs'!B17,2),0)</f>
+        <v>24</v>
       </c>
       <c r="C23" s="8" t="s">
         <v>13</v>
@@ -2007,7 +2007,7 @@
       </c>
       <c r="B24" s="14">
         <f>'User Inputs'!B16*'User Inputs'!B18*B23/8/1024</f>
-        <v>65.078125</v>
+        <v>91.875</v>
       </c>
       <c r="C24" s="8" t="s">
         <v>25</v>
@@ -2019,7 +2019,7 @@
       </c>
       <c r="B25" s="10">
         <f>'User Inputs'!B22</f>
-        <v>64</v>
+        <v>128</v>
       </c>
       <c r="C25" s="8" t="s">
         <v>25</v>
@@ -2031,7 +2031,7 @@
       </c>
       <c r="B26" s="16" t="str">
         <f>IF(B24&lt;=B25,"Fits","Overflow")</f>
-        <v>Overflow</v>
+        <v>Fits</v>
       </c>
       <c r="C26" s="8"/>
     </row>
@@ -2235,15 +2235,15 @@
     <row r="18" spans="1:4" ht="19.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="23">
         <f>'Performance Estimation'!B24</f>
-        <v>65.078125</v>
+        <v>91.875</v>
       </c>
       <c r="B18" s="23">
         <f>'Performance Estimation'!B25</f>
-        <v>64</v>
+        <v>128</v>
       </c>
       <c r="C18" s="24" t="str">
         <f>IF('Performance Estimation'!B26="Fits","✓ Fits","❌ Overflow")</f>
-        <v>❌ Overflow</v>
+        <v>✓ Fits</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="19.55" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>